<commit_message>
Add crawl imports and deepen V18-compatible audits
</commit_message>
<xml_diff>
--- a/exports/Kakawa_Chocolates_Enterprise_SEO_Package_v19/01_Evidence_and_Audits/Kakawa_Enterprise_SEO_Audit_v19.xlsx
+++ b/exports/Kakawa_Chocolates_Enterprise_SEO_Package_v19/01_Evidence_and_Audits/Kakawa_Enterprise_SEO_Audit_v19.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive" sheetId="1" r:id="R853c1d3eee894466"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Coverage" sheetId="2" r:id="R488cd63e43cb4180"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issue Register" sheetId="3" r:id="Ra3270ef3b04c4de4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Index" sheetId="4" r:id="Rfd9c371504ac45ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Page Inventory" sheetId="5" r:id="R5dc6f06873ec4204"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Rules" sheetId="6" r:id="Ra1098d9d5eae4215"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="7" r:id="R2e16de659cb04c48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive" sheetId="1" r:id="Raff502a2d25a4b39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Coverage" sheetId="2" r:id="R8e83209974bd4968"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issue Register" sheetId="3" r:id="Rceef4621620445c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Index" sheetId="4" r:id="Rf695131caf7f4f7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Page Inventory" sheetId="5" r:id="Rc0ee9edea32f4379"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Rules" sheetId="6" r:id="R13b25151be934fe6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="7" r:id="Rfe7f10704f384b83"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -277,7 +277,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rddf0cd6280884c70"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rad0f4ccbf2a14ab1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -784,7 +784,7 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3152044de5a4479"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f6c93fd622f4303"/>
 </x:worksheet>
 </file>
 
@@ -1065,7 +1065,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96652bb9055a4e91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R212bfef13c4d427c"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -1388,7 +1388,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14354164c3124c80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c827981a3f44f7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2548,7 +2548,7 @@
         <x:v>page_observation</x:v>
       </x:c>
       <x:c r="D39" t="str">
-        <x:v>HTTP 200; title=Wholesale Enquiries – Kakawa Chocolates Wholesale; meta=present; H1=Wholesale Chocolates | ; internal_links=35</x:v>
+        <x:v>HTTP 200; title=Wholesale Enquiries – Kakawa Chocolates Wholesale; meta=present; H1=Wholesale Chocolates; internal_links=35</x:v>
       </x:c>
       <x:c r="E39" t="str">
         <x:v>https://kakawachocolates.com.au/pages/wholesale</x:v>
@@ -9492,7 +9492,7 @@
         <x:v>page_observation</x:v>
       </x:c>
       <x:c r="D256" t="str">
-        <x:v>HTTP 200; title=Mother’s Day handcrafted flower chocolates – Kakawa Chocolates; meta=present; H1=Mother’s Day surprise with handcrafted flower chocolates | ; internal_links=44</x:v>
+        <x:v>HTTP 200; title=Mother’s Day handcrafted flower chocolates – Kakawa Chocolates; meta=present; H1=Mother’s Day surprise with handcrafted flower chocolates; internal_links=44</x:v>
       </x:c>
       <x:c r="E256" t="str">
         <x:v>https://kakawachocolates.com.au/blogs/chocolates/mother-s-day-surprise-with-handcrafted-flower-chocolates</x:v>
@@ -13138,7 +13138,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c76737d446a4aa3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20b70022753f4a13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14340,7 +14340,7 @@
         <x:v>Wholesale Enquiries – Kakawa Chocolates Wholesale</x:v>
       </x:c>
       <x:c r="F39" t="str">
-        <x:v>Wholesale Chocolates | </x:v>
+        <x:v>Wholesale Chocolates</x:v>
       </x:c>
       <x:c r="G39" t="str">
         <x:v>https://kakawachocolates.com.au/pages/wholesale</x:v>
@@ -21501,7 +21501,7 @@
         <x:v>Mother’s Day handcrafted flower chocolates – Kakawa Chocolates</x:v>
       </x:c>
       <x:c r="F256" t="str">
-        <x:v>Mother’s Day surprise with handcrafted flower chocolates | </x:v>
+        <x:v>Mother’s Day surprise with handcrafted flower chocolates</x:v>
       </x:c>
       <x:c r="G256" t="str">
         <x:v>https://kakawachocolates.com.au/blogs/chocolates/mother-s-day-surprise-with-handcrafted-flower-chocolates</x:v>
@@ -25022,7 +25022,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c1df20206ad427f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3331d16b4f5a454c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25328,7 +25328,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5ad3183b50141ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2281b43cb204c57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25438,10 +25438,10 @@
         <x:v>Canonical actions</x:v>
       </x:c>
       <x:c r="B8" t="n">
-        <x:v>16</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C8" t="n">
-        <x:v>16</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D8" t="str">
         <x:v>PASS</x:v>
@@ -25458,10 +25458,10 @@
         <x:v>Content assets</x:v>
       </x:c>
       <x:c r="B9" t="n">
-        <x:v>6</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C9" t="n">
-        <x:v>6</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D9" t="str">
         <x:v>PASS</x:v>
@@ -25520,7 +25520,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6105dd0e3fed49ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re713823069024553"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>